<commit_message>
fix: PNG bounds, Nim import/keyword, .exe skip in read phase across all languages
- Rust: fix PNG IEND offset pos+8 (was pos+12), skip .exe from read count
- Go: fix PNG IEND offset pos+8 with bounds check
- Nim: fix PNG IEND offset pos+8, add sequtils import, rename 'new' var,
      skip .exe from read count, fix indentation
- C, C++: skip .exe from read count
</commit_message>
<xml_diff>
--- a/go/creeper/planilla.xlsx
+++ b/go/creeper/planilla.xlsx
@@ -54,4 +54,11 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=creeper_infection/.creeper_marker.txt>CREEPER VIRUS - INFECTION MARKER
+Timestamp: 2026-07-09 14:31:31
+Original file: planilla.xlsx
+This file was infected by the Creeper educational virus.
+
 </file>
</xml_diff>

<commit_message>
chore: limpieza completa + README global
- Limpia todos los directorios creeper/ (elimina infection.log, RTL clones, .exe, .o)
- Regenera 12 archivos de usuario limpios en cada directorio
- Agrega .gitignore (__pycache__, *.exe, infection.log, *.o)
- Elimina docs/docs.md obsoleto, docs/ vacío
- Elimina rust/access direct/ (directorio huérfano)
- README.md completo con instrucciones en español para los 6 lenguajes
</commit_message>
<xml_diff>
--- a/go/creeper/planilla.xlsx
+++ b/go/creeper/planilla.xlsx
@@ -54,11 +54,4 @@
     </row>
   </sheetData>
 </worksheet>
-</file>
-
-<file path=creeper_infection/.creeper_marker.txt>CREEPER VIRUS - INFECTION MARKER
-Timestamp: 2026-07-09 14:31:31
-Original file: planilla.xlsx
-This file was infected by the Creeper educational virus.
-
 </file>
</xml_diff>